<commit_message>
This is the updated file
</commit_message>
<xml_diff>
--- a/12603996.xlsx
+++ b/12603996.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://lpuin-my.sharepoint.com/personal/shubham_bither2026_lpu_in/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://lpuin-my.sharepoint.com/personal/shubham_bither2026_lpu_in/Documents/LPU/CAP776/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="129" documentId="8_{04F8DF2E-49C5-3B44-B164-C4F738DF63B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EE28A8C9-7262-4879-B4CA-CDBA3F7C5AE3}"/>
+  <xr:revisionPtr revIDLastSave="225" documentId="8_{04F8DF2E-49C5-3B44-B164-C4F738DF63B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E868EE42-802F-4A5F-924E-C3F03515BB48}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="81">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -257,6 +257,27 @@
   </si>
   <si>
     <t xml:space="preserve">tried to study but there was light cut off </t>
+  </si>
+  <si>
+    <t>because power cut issue I had to eat from macDonalds</t>
+  </si>
+  <si>
+    <t>power cut is effecting my productivity</t>
+  </si>
+  <si>
+    <t>today's day was good and I studies good today</t>
+  </si>
+  <si>
+    <t xml:space="preserve">went home for rakshabandhan on bike </t>
+  </si>
+  <si>
+    <t>received good news about my brother marriage</t>
+  </si>
+  <si>
+    <t>travel to room from home , extreme pain started in my injured lower back</t>
+  </si>
+  <si>
+    <t>my got fixed today after a month , when I shifted In room</t>
   </si>
 </sst>
 </file>
@@ -1499,176 +1520,354 @@
         <v>73</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A16" s="13"/>
-      <c r="B16" s="14"/>
-      <c r="C16" s="14"/>
-      <c r="D16" s="14"/>
-      <c r="E16" s="14"/>
-      <c r="F16" s="14"/>
-      <c r="G16" s="14"/>
-      <c r="H16" s="14"/>
-      <c r="I16" s="15" t="str">
+    <row r="16" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A16" s="13">
+        <v>46259</v>
+      </c>
+      <c r="B16" s="14">
+        <v>330</v>
+      </c>
+      <c r="C16" s="14">
+        <v>35</v>
+      </c>
+      <c r="D16" s="14">
+        <v>45</v>
+      </c>
+      <c r="E16" s="14">
+        <v>50</v>
+      </c>
+      <c r="F16" s="14">
+        <v>350</v>
+      </c>
+      <c r="G16" s="14">
+        <v>7</v>
+      </c>
+      <c r="H16" s="14">
+        <v>250</v>
+      </c>
+      <c r="I16" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J16" s="15" t="str">
+        <v>1060</v>
+      </c>
+      <c r="J16" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K16" s="16"/>
-      <c r="L16" s="16"/>
-      <c r="M16" s="16"/>
-      <c r="N16" s="17"/>
-    </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A17" s="13"/>
-      <c r="B17" s="14"/>
-      <c r="C17" s="14"/>
-      <c r="D17" s="14"/>
-      <c r="E17" s="14"/>
-      <c r="F17" s="14"/>
-      <c r="G17" s="14"/>
-      <c r="H17" s="14"/>
-      <c r="I17" s="15" t="str">
+        <v>380</v>
+      </c>
+      <c r="K16" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="L16" s="16" t="s">
+        <v>68</v>
+      </c>
+      <c r="M16" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="N16" s="17" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A17" s="13">
+        <v>46260</v>
+      </c>
+      <c r="B17" s="14">
+        <v>330</v>
+      </c>
+      <c r="C17" s="14">
+        <v>70</v>
+      </c>
+      <c r="D17" s="14">
+        <v>150</v>
+      </c>
+      <c r="E17" s="14">
+        <v>50</v>
+      </c>
+      <c r="F17" s="14">
+        <v>200</v>
+      </c>
+      <c r="G17" s="14">
+        <v>4</v>
+      </c>
+      <c r="H17" s="14">
+        <v>360</v>
+      </c>
+      <c r="I17" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J17" s="15" t="str">
+        <v>1160</v>
+      </c>
+      <c r="J17" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K17" s="16"/>
-      <c r="L17" s="16"/>
-      <c r="M17" s="16"/>
-      <c r="N17" s="17"/>
-    </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A18" s="13"/>
-      <c r="B18" s="14"/>
-      <c r="C18" s="14"/>
-      <c r="D18" s="14"/>
-      <c r="E18" s="14"/>
-      <c r="F18" s="14"/>
-      <c r="G18" s="14"/>
-      <c r="H18" s="14"/>
-      <c r="I18" s="15" t="str">
+        <v>280</v>
+      </c>
+      <c r="K17" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="L17" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="M17" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N17" s="17" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A18" s="13">
+        <v>46261</v>
+      </c>
+      <c r="B18" s="14">
+        <v>330</v>
+      </c>
+      <c r="C18" s="14">
+        <v>80</v>
+      </c>
+      <c r="D18" s="14">
+        <v>200</v>
+      </c>
+      <c r="E18" s="14">
+        <v>50</v>
+      </c>
+      <c r="F18" s="14">
+        <v>350</v>
+      </c>
+      <c r="G18" s="14">
+        <v>7</v>
+      </c>
+      <c r="H18" s="14">
+        <v>230</v>
+      </c>
+      <c r="I18" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J18" s="15" t="str">
+        <v>1240</v>
+      </c>
+      <c r="J18" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K18" s="16"/>
-      <c r="L18" s="16"/>
-      <c r="M18" s="16"/>
-      <c r="N18" s="17"/>
-    </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A19" s="13"/>
-      <c r="B19" s="14"/>
-      <c r="C19" s="14"/>
-      <c r="D19" s="14"/>
-      <c r="E19" s="14"/>
-      <c r="F19" s="14"/>
-      <c r="G19" s="14"/>
-      <c r="H19" s="14"/>
-      <c r="I19" s="15" t="str">
+        <v>200</v>
+      </c>
+      <c r="K18" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L18" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M18" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N18" s="17" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A19" s="13">
+        <v>46262</v>
+      </c>
+      <c r="B19" s="14">
+        <v>360</v>
+      </c>
+      <c r="C19" s="14">
+        <v>70</v>
+      </c>
+      <c r="D19" s="14">
+        <v>0</v>
+      </c>
+      <c r="E19" s="14">
+        <v>0</v>
+      </c>
+      <c r="F19" s="14">
+        <v>100</v>
+      </c>
+      <c r="G19" s="14">
+        <v>2</v>
+      </c>
+      <c r="H19" s="14">
+        <v>300</v>
+      </c>
+      <c r="I19" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J19" s="15" t="str">
+        <v>830</v>
+      </c>
+      <c r="J19" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K19" s="16"/>
-      <c r="L19" s="16"/>
-      <c r="M19" s="16"/>
-      <c r="N19" s="17"/>
-    </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A20" s="13"/>
-      <c r="B20" s="14"/>
-      <c r="C20" s="14"/>
-      <c r="D20" s="14"/>
-      <c r="E20" s="14"/>
-      <c r="F20" s="14"/>
-      <c r="G20" s="14"/>
-      <c r="H20" s="14"/>
-      <c r="I20" s="15" t="str">
+        <v>610</v>
+      </c>
+      <c r="K19" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="L19" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="M19" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="N19" s="17" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A20" s="13">
+        <v>46263</v>
+      </c>
+      <c r="B20" s="14">
+        <v>540</v>
+      </c>
+      <c r="C20" s="14">
+        <v>0</v>
+      </c>
+      <c r="D20" s="14">
+        <v>170</v>
+      </c>
+      <c r="E20" s="14">
+        <v>0</v>
+      </c>
+      <c r="F20" s="14">
+        <v>0</v>
+      </c>
+      <c r="G20" s="14">
+        <v>0</v>
+      </c>
+      <c r="H20" s="14">
+        <v>430</v>
+      </c>
+      <c r="I20" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J20" s="15" t="str">
+        <v>1140</v>
+      </c>
+      <c r="J20" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K20" s="16"/>
-      <c r="L20" s="16"/>
-      <c r="M20" s="16"/>
-      <c r="N20" s="17"/>
-    </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A21" s="13"/>
-      <c r="B21" s="14"/>
-      <c r="C21" s="14"/>
-      <c r="D21" s="14"/>
-      <c r="E21" s="14"/>
-      <c r="F21" s="14"/>
-      <c r="G21" s="14"/>
-      <c r="H21" s="14"/>
-      <c r="I21" s="15" t="str">
+        <v>300</v>
+      </c>
+      <c r="K20" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="L20" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="M20" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N20" s="17" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A21" s="13">
+        <v>46264</v>
+      </c>
+      <c r="B21" s="14">
+        <v>360</v>
+      </c>
+      <c r="C21" s="14">
+        <v>45</v>
+      </c>
+      <c r="D21" s="14">
+        <v>0</v>
+      </c>
+      <c r="E21" s="14">
+        <v>0</v>
+      </c>
+      <c r="F21" s="14">
+        <v>0</v>
+      </c>
+      <c r="G21" s="14">
+        <v>0</v>
+      </c>
+      <c r="H21" s="14">
+        <v>600</v>
+      </c>
+      <c r="I21" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J21" s="15" t="str">
+        <v>1005</v>
+      </c>
+      <c r="J21" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K21" s="16"/>
-      <c r="L21" s="16"/>
-      <c r="M21" s="16"/>
-      <c r="N21" s="17"/>
-    </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A22" s="13"/>
-      <c r="B22" s="14"/>
-      <c r="C22" s="14"/>
-      <c r="D22" s="14"/>
-      <c r="E22" s="14"/>
-      <c r="F22" s="14"/>
-      <c r="G22" s="14"/>
-      <c r="H22" s="14"/>
-      <c r="I22" s="15" t="str">
+        <v>435</v>
+      </c>
+      <c r="K21" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="L21" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="M21" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="N21" s="17" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A22" s="13">
+        <v>46265</v>
+      </c>
+      <c r="B22" s="14">
+        <v>390</v>
+      </c>
+      <c r="C22" s="14">
+        <v>80</v>
+      </c>
+      <c r="D22" s="14">
+        <v>220</v>
+      </c>
+      <c r="E22" s="14">
+        <v>45</v>
+      </c>
+      <c r="F22" s="14">
+        <v>100</v>
+      </c>
+      <c r="G22" s="14">
+        <v>2</v>
+      </c>
+      <c r="H22" s="14">
+        <v>450</v>
+      </c>
+      <c r="I22" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J22" s="15" t="str">
+        <v>1285</v>
+      </c>
+      <c r="J22" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K22" s="16"/>
-      <c r="L22" s="16"/>
-      <c r="M22" s="16"/>
-      <c r="N22" s="17"/>
+        <v>155</v>
+      </c>
+      <c r="K22" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L22" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M22" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N22" s="17" t="s">
+        <v>80</v>
+      </c>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A23" s="13"/>
-      <c r="B23" s="14"/>
-      <c r="C23" s="14"/>
+      <c r="A23" s="13">
+        <v>46266</v>
+      </c>
+      <c r="B23" s="14">
+        <v>330</v>
+      </c>
+      <c r="C23" s="14">
+        <v>45</v>
+      </c>
       <c r="D23" s="14"/>
       <c r="E23" s="14"/>
-      <c r="F23" s="14"/>
-      <c r="G23" s="14"/>
+      <c r="F23" s="14">
+        <v>6</v>
+      </c>
+      <c r="G23" s="14">
+        <v>300</v>
+      </c>
       <c r="H23" s="14"/>
-      <c r="I23" s="15" t="str">
+      <c r="I23" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J23" s="15" t="str">
+        <v>381</v>
+      </c>
+      <c r="J23" s="15">
         <f t="shared" si="1"/>
-        <v/>
+        <v>1059</v>
       </c>
       <c r="K23" s="16"/>
       <c r="L23" s="16"/>

</xml_diff>

<commit_message>
This is the updated version
</commit_message>
<xml_diff>
--- a/12603996.xlsx
+++ b/12603996.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://lpuin-my.sharepoint.com/personal/shubham_bither2026_lpu_in/Documents/CAP776/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="232" documentId="8_{04F8DF2E-49C5-3B44-B164-C4F738DF63B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{76272874-9A33-46CB-AE48-27661DEDFBC0}"/>
+  <xr:revisionPtr revIDLastSave="241" documentId="8_{04F8DF2E-49C5-3B44-B164-C4F738DF63B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{435497CD-0C58-4126-B6D6-B7AF058A852A}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -561,6 +561,10 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -1858,21 +1862,21 @@
         <v>50</v>
       </c>
       <c r="F23" s="14">
+        <v>300</v>
+      </c>
+      <c r="G23" s="14">
         <v>6</v>
-      </c>
-      <c r="G23" s="14">
-        <v>300</v>
       </c>
       <c r="H23" s="14">
         <v>360</v>
       </c>
       <c r="I23" s="15">
         <f t="shared" si="0"/>
-        <v>851</v>
+        <v>1145</v>
       </c>
       <c r="J23" s="15">
         <f t="shared" si="1"/>
-        <v>589</v>
+        <v>295</v>
       </c>
       <c r="K23" s="16" t="s">
         <v>61</v>
@@ -1888,21 +1892,31 @@
       </c>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A24" s="13"/>
-      <c r="B24" s="14"/>
-      <c r="C24" s="14"/>
+      <c r="A24" s="13">
+        <v>46267</v>
+      </c>
+      <c r="B24" s="14">
+        <v>390</v>
+      </c>
+      <c r="C24" s="14">
+        <v>80</v>
+      </c>
       <c r="D24" s="14"/>
       <c r="E24" s="14"/>
-      <c r="F24" s="14"/>
-      <c r="G24" s="14"/>
+      <c r="F24" s="14">
+        <v>20</v>
+      </c>
+      <c r="G24" s="14">
+        <v>4</v>
+      </c>
       <c r="H24" s="14"/>
-      <c r="I24" s="15" t="str">
+      <c r="I24" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J24" s="15" t="str">
+        <v>490</v>
+      </c>
+      <c r="J24" s="15">
         <f t="shared" si="1"/>
-        <v/>
+        <v>950</v>
       </c>
       <c r="K24" s="16"/>
       <c r="L24" s="16"/>

</xml_diff>

<commit_message>
Updated after 2 days
</commit_message>
<xml_diff>
--- a/12603996.xlsx
+++ b/12603996.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://lpuin-my.sharepoint.com/personal/shubham_bither2026_lpu_in/Documents/CAP776/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="272" documentId="8_{04F8DF2E-49C5-3B44-B164-C4F738DF63B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{47BF56F8-DB77-470A-9ED0-73E43DF1CF91}"/>
+  <xr:revisionPtr revIDLastSave="310" documentId="8_{04F8DF2E-49C5-3B44-B164-C4F738DF63B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E11131B0-166E-41E9-9037-BCCC2B4166DE}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="88">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -290,6 +290,15 @@
   </si>
   <si>
     <t xml:space="preserve">went home on bike at night , new experience </t>
+  </si>
+  <si>
+    <t>studied for first CA</t>
+  </si>
+  <si>
+    <t>even after riding 120 km on bike I still fill energized</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ca was good , question level was medium </t>
   </si>
 </sst>
 </file>
@@ -1917,7 +1926,7 @@
         <v>120</v>
       </c>
       <c r="F24" s="14">
-        <v>20</v>
+        <v>200</v>
       </c>
       <c r="G24" s="14">
         <v>4</v>
@@ -1927,11 +1936,11 @@
       </c>
       <c r="I24" s="15">
         <f t="shared" si="0"/>
-        <v>1130</v>
+        <v>1310</v>
       </c>
       <c r="J24" s="15">
         <f t="shared" si="1"/>
-        <v>310</v>
+        <v>130</v>
       </c>
       <c r="K24" s="16" t="s">
         <v>64</v>
@@ -2039,70 +2048,142 @@
       </c>
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A27" s="13"/>
-      <c r="B27" s="14"/>
-      <c r="C27" s="14"/>
-      <c r="D27" s="14"/>
-      <c r="E27" s="14"/>
-      <c r="F27" s="14"/>
-      <c r="G27" s="14"/>
-      <c r="H27" s="14"/>
-      <c r="I27" s="15" t="str">
+      <c r="A27" s="13">
+        <v>46270</v>
+      </c>
+      <c r="B27" s="14">
+        <v>540</v>
+      </c>
+      <c r="C27" s="14">
+        <v>70</v>
+      </c>
+      <c r="D27" s="14">
+        <v>120</v>
+      </c>
+      <c r="E27" s="14">
+        <v>0</v>
+      </c>
+      <c r="F27" s="14">
+        <v>0</v>
+      </c>
+      <c r="G27" s="14">
+        <v>0</v>
+      </c>
+      <c r="H27" s="14">
+        <v>545</v>
+      </c>
+      <c r="I27" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J27" s="15" t="str">
+        <v>1275</v>
+      </c>
+      <c r="J27" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K27" s="16"/>
-      <c r="L27" s="16"/>
-      <c r="M27" s="16"/>
-      <c r="N27" s="17"/>
-    </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A28" s="13"/>
-      <c r="B28" s="14"/>
-      <c r="C28" s="14"/>
-      <c r="D28" s="14"/>
-      <c r="E28" s="14"/>
-      <c r="F28" s="14"/>
-      <c r="G28" s="14"/>
-      <c r="H28" s="14"/>
-      <c r="I28" s="15" t="str">
+        <v>165</v>
+      </c>
+      <c r="K27" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L27" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="M27" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N27" s="17" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="28" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A28" s="13">
+        <v>46271</v>
+      </c>
+      <c r="B28" s="14">
+        <v>540</v>
+      </c>
+      <c r="C28" s="14">
+        <v>120</v>
+      </c>
+      <c r="D28" s="14">
+        <v>145</v>
+      </c>
+      <c r="E28" s="14">
+        <v>0</v>
+      </c>
+      <c r="F28" s="14">
+        <v>0</v>
+      </c>
+      <c r="G28" s="14">
+        <v>0</v>
+      </c>
+      <c r="H28" s="14">
+        <v>220</v>
+      </c>
+      <c r="I28" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J28" s="15" t="str">
+        <v>1025</v>
+      </c>
+      <c r="J28" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K28" s="16"/>
-      <c r="L28" s="16"/>
-      <c r="M28" s="16"/>
-      <c r="N28" s="17"/>
-    </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A29" s="13"/>
-      <c r="B29" s="14"/>
-      <c r="C29" s="14"/>
-      <c r="D29" s="14"/>
-      <c r="E29" s="14"/>
-      <c r="F29" s="14"/>
-      <c r="G29" s="14"/>
-      <c r="H29" s="14"/>
-      <c r="I29" s="15" t="str">
+        <v>415</v>
+      </c>
+      <c r="K28" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L28" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M28" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="N28" s="17" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="29" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A29" s="13">
+        <v>46272</v>
+      </c>
+      <c r="B29" s="14">
+        <v>360</v>
+      </c>
+      <c r="C29" s="14">
+        <v>80</v>
+      </c>
+      <c r="D29" s="14">
+        <v>240</v>
+      </c>
+      <c r="E29" s="14">
+        <v>210</v>
+      </c>
+      <c r="F29" s="14">
+        <v>200</v>
+      </c>
+      <c r="G29" s="14">
+        <v>4</v>
+      </c>
+      <c r="H29" s="14">
+        <v>350</v>
+      </c>
+      <c r="I29" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J29" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J29" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K29" s="16"/>
-      <c r="L29" s="16"/>
-      <c r="M29" s="16"/>
-      <c r="N29" s="17"/>
+        <v>0</v>
+      </c>
+      <c r="K29" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="L29" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="M29" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N29" s="17" t="s">
+        <v>87</v>
+      </c>
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A30" s="13"/>

</xml_diff>

<commit_message>
Updated for two days
</commit_message>
<xml_diff>
--- a/12603996.xlsx
+++ b/12603996.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://lpuin-my.sharepoint.com/personal/shubham_bither2026_lpu_in/Documents/CAP776/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="350" documentId="8_{04F8DF2E-49C5-3B44-B164-C4F738DF63B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A04024F9-42A2-49EB-882C-47F58D652C1F}"/>
+  <xr:revisionPtr revIDLastSave="375" documentId="8_{04F8DF2E-49C5-3B44-B164-C4F738DF63B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CE09EABE-76A7-4171-904F-1E909C6481DD}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="93">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -308,6 +308,12 @@
   </si>
   <si>
     <t xml:space="preserve">didn't attend freshers party </t>
+  </si>
+  <si>
+    <t>arrived at home , joined training classes</t>
+  </si>
+  <si>
+    <t>started studying late due to headache</t>
   </si>
 </sst>
 </file>
@@ -2332,49 +2338,97 @@
         <v>90</v>
       </c>
     </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A33" s="13"/>
-      <c r="B33" s="14"/>
-      <c r="C33" s="14"/>
-      <c r="D33" s="14"/>
-      <c r="E33" s="14"/>
-      <c r="F33" s="14"/>
-      <c r="G33" s="14"/>
-      <c r="H33" s="14"/>
-      <c r="I33" s="15" t="str">
+    <row r="33" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A33" s="13">
+        <v>46276</v>
+      </c>
+      <c r="B33" s="14">
+        <v>300</v>
+      </c>
+      <c r="C33" s="14">
+        <v>100</v>
+      </c>
+      <c r="D33" s="14">
+        <v>0</v>
+      </c>
+      <c r="E33" s="14">
+        <v>0</v>
+      </c>
+      <c r="F33" s="14">
+        <v>250</v>
+      </c>
+      <c r="G33" s="14">
+        <v>5</v>
+      </c>
+      <c r="H33" s="14">
+        <v>630</v>
+      </c>
+      <c r="I33" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J33" s="15" t="str">
+        <v>1280</v>
+      </c>
+      <c r="J33" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K33" s="16"/>
-      <c r="L33" s="16"/>
-      <c r="M33" s="16"/>
-      <c r="N33" s="17"/>
-    </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A34" s="13"/>
-      <c r="B34" s="14"/>
-      <c r="C34" s="14"/>
-      <c r="D34" s="14"/>
-      <c r="E34" s="14"/>
-      <c r="F34" s="14"/>
-      <c r="G34" s="14"/>
-      <c r="H34" s="14"/>
-      <c r="I34" s="15" t="str">
+        <v>160</v>
+      </c>
+      <c r="K33" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="L33" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="M33" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N33" s="17" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="34" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A34" s="13">
+        <v>46277</v>
+      </c>
+      <c r="B34" s="14">
+        <v>600</v>
+      </c>
+      <c r="C34" s="14">
+        <v>25</v>
+      </c>
+      <c r="D34" s="14">
+        <v>200</v>
+      </c>
+      <c r="E34" s="14">
+        <v>75</v>
+      </c>
+      <c r="F34" s="14">
+        <v>0</v>
+      </c>
+      <c r="G34" s="14">
+        <v>0</v>
+      </c>
+      <c r="H34" s="14">
+        <v>540</v>
+      </c>
+      <c r="I34" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J34" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J34" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K34" s="16"/>
-      <c r="L34" s="16"/>
-      <c r="M34" s="16"/>
-      <c r="N34" s="17"/>
+        <v>0</v>
+      </c>
+      <c r="K34" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="L34" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="M34" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N34" s="17" t="s">
+        <v>92</v>
+      </c>
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A35" s="13"/>

</xml_diff>